<commit_message>
Remove legacy script and update Excel processing for ECG denoising
- Deleted the outdated script `update_records_list_adding_ml_noises_v6.py` which was no longer needed.
- Modified the Excel processing logic to remove legacy columns (`ml_nz_cnt`, `ml_nz_len`) and replaced them with new output columns (`out`, `rdr`, `noi`).
- Updated the calculation of `ml_nz_frac%` to directly use `tp%` from the denoising statistics.
- Ensured that the denoising pipeline is prepared once before processing the main loop for efficiency.
- Adjusted the handling of JSON metadata and data files to reflect the new structure and requirements.
</commit_message>
<xml_diff>
--- a/0_SELECT_ZIVE_DATA_2023/AtsisiuntimasZiveDuomenu/DuomenysTestui/zive_irasai_testui.xlsx
+++ b/0_SELECT_ZIVE_DATA_2023/AtsisiuntimasZiveDuomenu/DuomenysTestui/zive_irasai_testui.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\kesju\DI\2025_ZIVEO\PROJECT_TRAIN_UNET\0_SELECT_ZIVE_DATA_2023\AtsisiuntimasZiveDuomenu\DuomenysTestui\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3671BBDB-C443-431D-B8DC-7730F9D8E424}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59DB5FE3-1156-46F4-A803-D44DF3C85BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="18600" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="600" yWindow="1140" windowWidth="18600" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="88">
   <si>
     <t>filename</t>
   </si>
@@ -286,6 +286,18 @@
   </si>
   <si>
     <t xml:space="preserve">Švarumo lygis didžojoje dalyje arti 10, tačiau apie vidurį yra ilgas fragmentas su nežymėtu silpnu# raumenų triukšmu. Žymėjimas koreguotas, dėl įtraukimo į mokymo grupę, abejotina </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> out</t>
+  </si>
+  <si>
+    <t>rdr</t>
+  </si>
+  <si>
+    <t>noi</t>
+  </si>
+  <si>
+    <t>tp%</t>
   </si>
 </sst>
 </file>
@@ -729,7 +741,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AE12"/>
+  <dimension ref="A1:AI12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="13.6328125" style="13" customWidth="1"/>
@@ -744,19 +756,19 @@
     <col min="16" max="16" width="4.90625" customWidth="1"/>
     <col min="17" max="17" width="8.90625" customWidth="1"/>
     <col min="18" max="18" width="9.26953125" customWidth="1"/>
-    <col min="19" max="19" width="9.7265625" style="9" customWidth="1"/>
-    <col min="20" max="20" width="9.81640625" customWidth="1"/>
-    <col min="21" max="21" width="13.1796875" customWidth="1"/>
-    <col min="22" max="22" width="12.08984375" style="10" customWidth="1"/>
-    <col min="23" max="23" width="54.6328125" customWidth="1"/>
-    <col min="24" max="24" width="28.81640625" customWidth="1"/>
-    <col min="25" max="25" width="27.1796875" customWidth="1"/>
-    <col min="26" max="31" width="13.6328125" style="5" customWidth="1"/>
-    <col min="32" max="32" width="13.6328125" customWidth="1"/>
-    <col min="33" max="48" width="8.7265625" customWidth="1"/>
+    <col min="19" max="23" width="9.7265625" style="9" customWidth="1"/>
+    <col min="24" max="24" width="9.81640625" customWidth="1"/>
+    <col min="25" max="25" width="13.1796875" customWidth="1"/>
+    <col min="26" max="26" width="12.08984375" style="10" customWidth="1"/>
+    <col min="27" max="27" width="54.6328125" customWidth="1"/>
+    <col min="28" max="28" width="28.81640625" customWidth="1"/>
+    <col min="29" max="29" width="27.1796875" customWidth="1"/>
+    <col min="30" max="35" width="13.6328125" style="5" customWidth="1"/>
+    <col min="36" max="36" width="13.6328125" customWidth="1"/>
+    <col min="37" max="52" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -815,28 +827,40 @@
         <v>77</v>
       </c>
       <c r="T1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="X1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="W1" s="11" t="s">
+      <c r="AA1" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>20</v>
       </c>
@@ -897,23 +921,35 @@
       <c r="U2" s="8">
         <v>0</v>
       </c>
-      <c r="V2" s="10">
-        <v>0</v>
-      </c>
-      <c r="W2" t="s">
+      <c r="V2" s="8">
+        <v>0</v>
+      </c>
+      <c r="W2" s="9">
+        <v>0</v>
+      </c>
+      <c r="X2" s="8">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="8">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA2" t="s">
         <v>60</v>
       </c>
-      <c r="X2" t="s">
+      <c r="AB2" t="s">
         <v>22</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="AC2" t="s">
         <v>21</v>
       </c>
-      <c r="Z2" s="5" t="s">
+      <c r="AD2" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>24</v>
       </c>
@@ -974,23 +1010,35 @@
       <c r="U3" s="8">
         <v>0</v>
       </c>
-      <c r="V3" s="10">
-        <v>0</v>
-      </c>
-      <c r="W3" t="s">
+      <c r="V3" s="8">
+        <v>0</v>
+      </c>
+      <c r="W3" s="9">
+        <v>0</v>
+      </c>
+      <c r="X3" s="8">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="8">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="s">
         <v>60</v>
       </c>
-      <c r="X3" t="s">
+      <c r="AB3" t="s">
         <v>25</v>
       </c>
-      <c r="Y3" t="s">
+      <c r="AC3" t="s">
         <v>21</v>
       </c>
-      <c r="Z3" s="5" t="s">
+      <c r="AD3" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>27</v>
       </c>
@@ -1051,23 +1099,35 @@
       <c r="U4" s="8">
         <v>0</v>
       </c>
-      <c r="V4" s="10">
-        <v>0</v>
-      </c>
-      <c r="W4" t="s">
+      <c r="V4" s="8">
+        <v>0</v>
+      </c>
+      <c r="W4" s="9">
+        <v>0</v>
+      </c>
+      <c r="X4" s="8">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="8">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="s">
         <v>61</v>
       </c>
-      <c r="X4" t="s">
+      <c r="AB4" t="s">
         <v>28</v>
       </c>
-      <c r="Y4" t="s">
+      <c r="AC4" t="s">
         <v>10</v>
       </c>
-      <c r="Z4" s="5" t="s">
+      <c r="AD4" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>30</v>
       </c>
@@ -1128,23 +1188,35 @@
       <c r="U5" s="8">
         <v>0</v>
       </c>
-      <c r="V5" s="10">
-        <v>0</v>
-      </c>
-      <c r="W5" t="s">
+      <c r="V5" s="8">
+        <v>0</v>
+      </c>
+      <c r="W5" s="9">
+        <v>0</v>
+      </c>
+      <c r="X5" s="8">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="8">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="s">
         <v>60</v>
       </c>
-      <c r="X5" t="s">
+      <c r="AB5" t="s">
         <v>31</v>
       </c>
-      <c r="Y5" t="s">
+      <c r="AC5" t="s">
         <v>10</v>
       </c>
-      <c r="Z5" s="5" t="s">
+      <c r="AD5" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>18</v>
       </c>
@@ -1205,23 +1277,35 @@
       <c r="U6" s="8">
         <v>0</v>
       </c>
-      <c r="V6" s="10">
-        <v>0</v>
-      </c>
-      <c r="W6" t="s">
+      <c r="V6" s="8">
+        <v>0</v>
+      </c>
+      <c r="W6" s="9">
+        <v>0</v>
+      </c>
+      <c r="X6" s="8">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="8">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="s">
         <v>61</v>
       </c>
-      <c r="X6" t="s">
+      <c r="AB6" t="s">
         <v>19</v>
       </c>
-      <c r="Y6" t="s">
+      <c r="AC6" t="s">
         <v>10</v>
       </c>
-      <c r="Z6" s="5" t="s">
+      <c r="AD6" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>33</v>
       </c>
@@ -1282,23 +1366,35 @@
       <c r="U7" s="8">
         <v>0</v>
       </c>
-      <c r="V7" s="10">
-        <v>0</v>
-      </c>
-      <c r="W7" t="s">
+      <c r="V7" s="8">
+        <v>0</v>
+      </c>
+      <c r="W7" s="9">
+        <v>0</v>
+      </c>
+      <c r="X7" s="8">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="8">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="s">
         <v>60</v>
       </c>
-      <c r="X7" t="s">
+      <c r="AB7" t="s">
         <v>34</v>
       </c>
-      <c r="Y7" t="s">
+      <c r="AC7" t="s">
         <v>10</v>
       </c>
-      <c r="Z7" s="6" t="s">
+      <c r="AD7" s="6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>16</v>
       </c>
@@ -1359,23 +1455,35 @@
       <c r="U8" s="8">
         <v>0</v>
       </c>
-      <c r="V8" s="10">
-        <v>0</v>
-      </c>
-      <c r="W8" t="s">
+      <c r="V8" s="8">
+        <v>0</v>
+      </c>
+      <c r="W8" s="9">
+        <v>0</v>
+      </c>
+      <c r="X8" s="8">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="8">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="s">
         <v>61</v>
       </c>
-      <c r="X8" t="s">
+      <c r="AB8" t="s">
         <v>17</v>
       </c>
-      <c r="Y8" t="s">
+      <c r="AC8" t="s">
         <v>10</v>
       </c>
-      <c r="Z8" s="5" t="s">
+      <c r="AD8" s="5" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>14</v>
       </c>
@@ -1436,20 +1544,32 @@
       <c r="U9" s="8">
         <v>0</v>
       </c>
-      <c r="V9" s="10">
-        <v>0</v>
-      </c>
-      <c r="W9" t="s">
+      <c r="V9" s="8">
+        <v>0</v>
+      </c>
+      <c r="W9" s="9">
+        <v>0</v>
+      </c>
+      <c r="X9" s="8">
+        <v>0</v>
+      </c>
+      <c r="Y9" s="8">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="s">
         <v>61</v>
       </c>
-      <c r="X9" t="s">
+      <c r="AB9" t="s">
         <v>15</v>
       </c>
-      <c r="Y9" t="s">
+      <c r="AC9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
@@ -1510,23 +1630,35 @@
       <c r="U10" s="8">
         <v>0</v>
       </c>
-      <c r="V10" s="10">
-        <v>0</v>
-      </c>
-      <c r="W10" t="s">
+      <c r="V10" s="8">
+        <v>0</v>
+      </c>
+      <c r="W10" s="9">
+        <v>0</v>
+      </c>
+      <c r="X10" s="8">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="8">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="s">
         <v>61</v>
       </c>
-      <c r="X10" t="s">
+      <c r="AB10" t="s">
         <v>11</v>
       </c>
-      <c r="Y10" t="s">
+      <c r="AC10" t="s">
         <v>10</v>
       </c>
-      <c r="Z10" s="5" t="s">
+      <c r="AD10" s="5" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
@@ -1587,20 +1719,32 @@
       <c r="U11" s="8">
         <v>0</v>
       </c>
-      <c r="V11" s="10">
-        <v>0</v>
-      </c>
-      <c r="W11" t="s">
+      <c r="V11" s="8">
+        <v>0</v>
+      </c>
+      <c r="W11" s="9">
+        <v>0</v>
+      </c>
+      <c r="X11" s="8">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="8">
+        <v>0</v>
+      </c>
+      <c r="Z11" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="s">
         <v>61</v>
       </c>
-      <c r="X11" t="s">
+      <c r="AB11" t="s">
         <v>13</v>
       </c>
-      <c r="Y11" t="s">
+      <c r="AC11" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>36</v>
       </c>
@@ -1661,21 +1805,33 @@
       <c r="U12" s="8">
         <v>0</v>
       </c>
-      <c r="V12" s="10">
-        <v>0</v>
-      </c>
-      <c r="W12" t="s">
+      <c r="V12" s="8">
+        <v>0</v>
+      </c>
+      <c r="W12" s="9">
+        <v>0</v>
+      </c>
+      <c r="X12" s="8">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="8">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="s">
         <v>61</v>
       </c>
-      <c r="X12" t="s">
+      <c r="AB12" t="s">
         <v>38</v>
       </c>
-      <c r="Y12" t="s">
+      <c r="AC12" t="s">
         <v>37</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Z12">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AD12">
     <sortCondition ref="A2:A12"/>
   </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add update_records_list_v5.py and update_records_list_v5.sh for processing ZIVE data
- Introduced update_records_list_v5.py: a directory-only version for updating records with ML noise statistics.
- Simplified column mapping and ensured noise fractions are always percentages.
- Added update_records_list_v5.sh for easy execution with example commands for testing and production use.
</commit_message>
<xml_diff>
--- a/0_SELECT_ZIVE_DATA_2023/AtsisiuntimasZiveDuomenu/DuomenysTestui/zive_irasai_testui.xlsx
+++ b/0_SELECT_ZIVE_DATA_2023/AtsisiuntimasZiveDuomenu/DuomenysTestui/zive_irasai_testui.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\kesju\DI\2025_ZIVEO\PROJECT_TRAIN_UNET\0_SELECT_ZIVE_DATA_2023\AtsisiuntimasZiveDuomenu\DuomenysTestui\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59DB5FE3-1156-46F4-A803-D44DF3C85BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE813F25-994B-4116-BCAF-AB9E2B24047A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="600" yWindow="1140" windowWidth="18600" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Zymejimas" sheetId="2" r:id="rId2"/>
+    <sheet name="Records" sheetId="1" r:id="rId1"/>
+    <sheet name="Parameters" sheetId="3" r:id="rId2"/>
+    <sheet name="Marks" sheetId="2" r:id="rId3"/>
+    <sheet name="Notes" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="89">
   <si>
     <t>filename</t>
   </si>
@@ -298,6 +300,9 @@
   </si>
   <si>
     <t>tp%</t>
+  </si>
+  <si>
+    <t>excl</t>
   </si>
 </sst>
 </file>
@@ -969,7 +974,7 @@
         <v>9999</v>
       </c>
       <c r="H3" t="s">
-        <v>8</v>
+        <v>88</v>
       </c>
       <c r="I3" s="8">
         <v>4850</v>
@@ -1058,7 +1063,7 @@
         <v>9999</v>
       </c>
       <c r="H4" t="s">
-        <v>8</v>
+        <v>88</v>
       </c>
       <c r="I4" s="8">
         <v>6018</v>
@@ -1840,6 +1845,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCB03E47-ABEC-4DDB-9DFB-2134085102CA}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6740BA52-0B9E-43BD-B693-6B53C9B815B0}">
   <dimension ref="B2:C15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1900,4 +1914,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5226947-0C6C-41DD-89DC-9E5D5CCC7401}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>